<commit_message>
Refresh week May 4-10 with full data
</commit_message>
<xml_diff>
--- a/driver statistics report/Driver Statistics Report ( 04 May 2026 - 10 May 2026 ).xlsx
+++ b/driver statistics report/Driver Statistics Report ( 04 May 2026 - 10 May 2026 ).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="47">
   <si>
     <t>Driver Name</t>
   </si>
@@ -130,10 +130,13 @@
     <t>3.8</t>
   </si>
   <si>
+    <t>3.4</t>
+  </si>
+  <si>
     <t>Commercial Vehicle</t>
   </si>
   <si>
-    <t>Driver Statistics Report (GZV4) (Generated 07 May 2026 15:10:01 MDT)</t>
+    <t>Driver Statistics Report (GZV4) (Generated 08 May 2026 13:32:21 MDT)</t>
   </si>
   <si>
     <t>Fleet: Fuelled Energy Marketing Inc</t>
@@ -566,7 +569,7 @@
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -583,7 +586,7 @@
     </row>
     <row r="2" spans="1:27">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -600,7 +603,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -617,7 +620,7 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -634,7 +637,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -651,7 +654,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -668,7 +671,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -914,7 +917,7 @@
         <v>0</v>
       </c>
       <c r="Z13" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -925,19 +928,19 @@
         <v>29</v>
       </c>
       <c r="D14" s="1">
-        <v>204</v>
+        <v>241</v>
       </c>
       <c r="E14" s="1">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="1">
-        <v>982</v>
+        <v>985</v>
       </c>
       <c r="H14" s="1">
-        <v>-18</v>
+        <v>-15</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>37</v>
@@ -991,10 +994,10 @@
         <v>0</v>
       </c>
       <c r="Z14" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AA14" s="1">
-        <v>-9</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -1071,7 +1074,7 @@
         <v>0</v>
       </c>
       <c r="Z15" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:27">
@@ -1082,25 +1085,25 @@
         <v>31</v>
       </c>
       <c r="D16" s="1">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="E16" s="1">
-        <v>0</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>35</v>
+        <v>53</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>969</v>
       </c>
       <c r="H16" s="1">
-        <v>0</v>
+        <v>-31</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J16" s="1">
-        <v>0</v>
+        <v>-18</v>
       </c>
       <c r="K16" s="1">
         <v>0</v>
@@ -1145,10 +1148,13 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Z16" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="AA16" s="1">
+        <v>-18</v>
       </c>
     </row>
     <row r="17" spans="1:27">
@@ -1159,7 +1165,7 @@
         <v>32</v>
       </c>
       <c r="D17" s="1">
-        <v>469</v>
+        <v>488</v>
       </c>
       <c r="E17" s="1">
         <v>75</v>
@@ -1225,7 +1231,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AA17" s="1">
         <v>-1</v>
@@ -1302,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="Z18" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:27">
@@ -1316,25 +1322,25 @@
         <v>35</v>
       </c>
       <c r="D19" s="1">
-        <v>673</v>
+        <v>831</v>
       </c>
       <c r="E19" s="1">
-        <v>72.95999999999999</v>
+        <v>70.52</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
       </c>
       <c r="G19" s="1">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="H19" s="1">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="I19" s="1">
-        <v>3.86</v>
+        <v>3.85</v>
       </c>
       <c r="J19" s="1">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="K19" s="1">
         <v>1</v>
@@ -1385,7 +1391,7 @@
         <v>35</v>
       </c>
       <c r="AA19" s="1">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace partial May 4-10 with full-week data, refresh feedback
</commit_message>
<xml_diff>
--- a/driver statistics report/Driver Statistics Report ( 04 May 2026 - 10 May 2026 ).xlsx
+++ b/driver statistics report/Driver Statistics Report ( 04 May 2026 - 10 May 2026 ).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
   <si>
     <t>Driver Name</t>
   </si>
@@ -127,16 +127,16 @@
     <t>0</t>
   </si>
   <si>
+    <t>3.7</t>
+  </si>
+  <si>
     <t>3.8</t>
   </si>
   <si>
-    <t>3.4</t>
-  </si>
-  <si>
     <t>Commercial Vehicle</t>
   </si>
   <si>
-    <t>Driver Statistics Report (GZV4) (Generated 08 May 2026 13:32:21 MDT)</t>
+    <t>Driver Statistics Report (GZV4) (Generated 11 May 2026 06:52:23 MDT)</t>
   </si>
   <si>
     <t>Fleet: Fuelled Energy Marketing Inc</t>
@@ -151,7 +151,7 @@
     <t>Caused By:  Other,Third party</t>
   </si>
   <si>
-    <t>Total Events:  1</t>
+    <t>Total Events:  3</t>
   </si>
   <si>
     <t>Note: The GreenZone Score and Total Impacts shown in this report are based on the user's current access permissions and may differ from the values displayed on the portal. The portal may reflect data for the entire fleet or a broader set of vehicles and drivers than what is available to the user</t>
@@ -851,28 +851,28 @@
         <v>28</v>
       </c>
       <c r="D13" s="1">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="E13" s="1">
-        <v>0</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>35</v>
+        <v>69</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>870</v>
       </c>
       <c r="H13" s="1">
-        <v>0</v>
+        <v>-130</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J13" s="1">
-        <v>0</v>
+        <v>-17</v>
       </c>
       <c r="K13" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" s="1">
         <v>0</v>
@@ -887,10 +887,10 @@
         <v>0</v>
       </c>
       <c r="P13" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="1">
-        <v>0</v>
+        <v>-79</v>
       </c>
       <c r="R13" s="1">
         <v>0</v>
@@ -918,6 +918,9 @@
       </c>
       <c r="Z13" s="1" t="s">
         <v>39</v>
+      </c>
+      <c r="AA13" s="1">
+        <v>-34</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -928,28 +931,28 @@
         <v>29</v>
       </c>
       <c r="D14" s="1">
-        <v>241</v>
+        <v>395</v>
       </c>
       <c r="E14" s="1">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="1">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="H14" s="1">
-        <v>-15</v>
+        <v>-13</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J14" s="1">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="K14" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" s="1">
         <v>0</v>
@@ -997,7 +1000,7 @@
         <v>39</v>
       </c>
       <c r="AA14" s="1">
-        <v>-6</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -1085,25 +1088,25 @@
         <v>31</v>
       </c>
       <c r="D16" s="1">
-        <v>102</v>
+        <v>316</v>
       </c>
       <c r="E16" s="1">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
       </c>
       <c r="G16" s="1">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="H16" s="1">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J16" s="1">
-        <v>-18</v>
+        <v>-20</v>
       </c>
       <c r="K16" s="1">
         <v>0</v>
@@ -1154,7 +1157,7 @@
         <v>39</v>
       </c>
       <c r="AA16" s="1">
-        <v>-18</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="17" spans="1:27">
@@ -1165,7 +1168,7 @@
         <v>32</v>
       </c>
       <c r="D17" s="1">
-        <v>488</v>
+        <v>664</v>
       </c>
       <c r="E17" s="1">
         <v>75</v>
@@ -1174,19 +1177,19 @@
         <v>0</v>
       </c>
       <c r="G17" s="1">
-        <v>991</v>
+        <v>976</v>
       </c>
       <c r="H17" s="1">
-        <v>-9</v>
+        <v>-24</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J17" s="1">
         <v>-8</v>
       </c>
       <c r="K17" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" s="1">
         <v>0</v>
@@ -1207,10 +1210,10 @@
         <v>0</v>
       </c>
       <c r="R17" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="1">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="T17" s="1">
         <v>0</v>
@@ -1225,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="X17" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y17" s="1">
         <v>0</v>
@@ -1234,7 +1237,7 @@
         <v>39</v>
       </c>
       <c r="AA17" s="1">
-        <v>-1</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="18" spans="1:27">
@@ -1322,52 +1325,52 @@
         <v>35</v>
       </c>
       <c r="D19" s="1">
-        <v>831</v>
+        <v>1560</v>
       </c>
       <c r="E19" s="1">
-        <v>70.52</v>
+        <v>70.83</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
       </c>
       <c r="G19" s="1">
-        <v>986</v>
+        <v>965</v>
       </c>
       <c r="H19" s="1">
-        <v>-14</v>
+        <v>-35</v>
       </c>
       <c r="I19" s="1">
-        <v>3.85</v>
+        <v>3.82</v>
       </c>
       <c r="J19" s="1">
+        <v>-12</v>
+      </c>
+      <c r="K19" s="1">
+        <v>3</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="1">
         <v>-10</v>
       </c>
-      <c r="K19" s="1">
+      <c r="R19" s="1">
         <v>1</v>
       </c>
-      <c r="L19" s="1">
-        <v>0</v>
-      </c>
-      <c r="M19" s="1">
-        <v>0</v>
-      </c>
-      <c r="N19" s="1">
-        <v>0</v>
-      </c>
-      <c r="O19" s="1">
-        <v>0</v>
-      </c>
-      <c r="P19" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>0</v>
-      </c>
-      <c r="R19" s="1">
-        <v>0</v>
-      </c>
       <c r="S19" s="1">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="T19" s="1">
         <v>0</v>
@@ -1382,16 +1385,16 @@
         <v>0</v>
       </c>
       <c r="X19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z19" s="1" t="s">
         <v>35</v>
       </c>
       <c r="AA19" s="1">
-        <v>-4</v>
+        <v>-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>